<commit_message>
change to https ab592da5e89406e94d2fe074e805e04c2e558455
</commit_message>
<xml_diff>
--- a/ig/update-vs-url/StructureDefinition-fr-core-ident-reliability.xlsx
+++ b/ig/update-vs-url/StructureDefinition-fr-core-ident-reliability.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-10-30T11:02:30+00:00</t>
+    <t>2023-11-06T10:17:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -336,7 +336,7 @@
     <t>required</t>
   </si>
   <si>
-    <t>http://hl7.fr/ig/fhir/core/ValueSet/fr-core-mode-validation-identite</t>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-mode-validation-identite</t>
   </si>
   <si>
     <t>base64Binary
@@ -677,7 +677,7 @@
     <col min="23" max="23" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="10.53125" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="1.04296875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="60.83203125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="61.78515625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="10.26171875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="42.03515625" customWidth="true" bestFit="true"/>

</xml_diff>